<commit_message>
Updated to correct issue with NAs from June and July 2025 suppression setting totals to 0. Also updated to remove timePeriod from earlier in the script as not used.
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{401B9959-841B-4BE2-9867-042A5800898B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACF0384-2D52-4FE0-B51C-D7107E9E5262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>November 2025 data</t>
   </si>
   <si>
-    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. The adjustment applied to the data has been calculated based on the average trend of the source data for the past year. As such, month-on-month trends during the affected period should be treated with caution.</t>
+    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. ONS suppressed some of the data in June and July 2025 due to quality concerns. As a result, the sum of new adverts across all SOCs may not equal the England total. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to reword caveats
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACF0384-2D52-4FE0-B51C-D7107E9E5262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38193FE4-DC94-4679-8579-1C9A195E03C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>November 2025 data</t>
   </si>
   <si>
-    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. ONS suppressed some of the data in June and July 2025 due to quality concerns. As a result, the sum of new adverts across all SOCs may not equal the England total. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
+    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. ONS have suppressed some of the data in June and July 2025 due to quality concerns. This has resulted in a drop in numbers over the months that include June and July 2025 in their rolling average calculation. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to apply the three-month rolling average calculation to the individual tables read in, rather than the final table. Update to add a banner to the dashboard notifying users of the switch to new adverts.
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38193FE4-DC94-4679-8579-1C9A195E03C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E80AAA4-229A-4894-A01C-A64D6313197E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>November 2025 data</t>
   </si>
   <si>
-    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. ONS have suppressed some of the data in June and July 2025 due to quality concerns. This has resulted in a drop in numbers over the months that include June and July 2025 in their rolling average calculation. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
+    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occured, only the unsuppressed data is included in the rolling average. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to caveats and to remove [x] line
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-2_dataText\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E80AAA4-229A-4894-A01C-A64D6313197E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3775556D-A6CF-46C1-85D4-568CAADE983A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -810,7 +810,7 @@
     <t>November 2025 data</t>
   </si>
   <si>
-    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occured, only the unsuppressed data is included in the rolling average. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
+    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occurred, only the data containing no suppression is included in the rolling average. ONS have partially imputed the data for October and November 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update national job ads summing NA error. Update job ads caveat text.
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C0C36F0-62C9-43FB-8465-A8623A0243A1}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7907F9B4-1A7A-4A91-B8DE-2231905DBF67}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -807,7 +807,7 @@
     <t>April 2026 data</t>
   </si>
   <si>
-    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occurred, only the data containing no suppression is included in the rolling average. ONS have partially imputed the data since October 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution. Additionally, a source of jobs was missing from the December 2025 and February 2026 data, and so some data has been suppressed in these months. Finally, March 2026 data is currently supressed so is excluded from any three-month averages.</t>
+    <t>These statistics should be treated as official statistics in development (previously known as experimental statistics). ONS have temporarily paused publication of the snapshot metric for online job adverts and so the dashboard currently shows the number of new adverts that have gone online in the month, presented as a three-month rolling average. The total across geographies may not sum to the England total. The data includes minor instances of suppression in June and July 2025 due to quality concerns. Where this has occurred, only the data containing no suppression is included in the rolling average. ONS have partially imputed the data since October 2025 in response to the source data presenting a larger level of duplicate adverts which are not being identified as such. As such, month-on-month trends during the affected period should be treated with caution. Additionally, a source of jobs was missing from the December 2025 and February 2026 data, and so some data has been suppressed in these months. Finally,  the entirety of the March 2026 data is currently supressed so is excluded from any three-month averages.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Bring in apprenticeship detail and add to dashboard. Still a few things remaining to fix (breakdown chart)
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D49753A-6234-4368-B01E-36E67032C381}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9250B018-2B86-44BF-9E5D-4DD6E1466454}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="230">
   <si>
     <t>inactiveRate</t>
   </si>
@@ -808,6 +808,47 @@
   </si>
   <si>
     <t>June 2026 data</t>
+  </si>
+  <si>
+    <t>apprenticeships</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator shows apprenticeship achievements. </t>
+  </si>
+  <si>
+    <t>Include all age apprenticeships.
+Apprenticeships are paid jobs that incorporate on-the-job and off-the-job training leading to nationally recognised qualifications.
+Achievements are the number of learners who successfully complete an individual aim in an academic year.</t>
+  </si>
+  <si>
+    <t>&lt;ol&gt;
+  &lt;li&gt;Total achievements is the count of learners that completed their qualification at any point during the stated academic period.&lt;/li&gt;
+ &lt;li&gt;Learners achieving more than one course will appear only once in the grand total.&lt;/li&gt;
+ &lt;li&gt;Years shown represent academic years.&lt;/li&gt;
+&lt;li&gt;Use caution when interpreting this data. A difference between subgroups does not necessarily imply any causality. There could be other contributing factors at work.&lt;/li&gt;
+&lt;li&gt;Figures for LSIP and CAs have been calculated from Local Authority District data to create a back series. There may be small differences to the published data for these geographies due to rounding errors.&lt;/li&gt;
+&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t>are apprenticeship volumes changing</t>
+  </si>
+  <si>
+    <t>The number of apprenticeships in</t>
+  </si>
+  <si>
+    <t>Apprenticeships</t>
+  </si>
+  <si>
+    <t>share of apprenticeships</t>
+  </si>
+  <si>
+    <t>Apprenticeships are</t>
+  </si>
+  <si>
+    <t>&lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/apprenticeships/2024-25'&gt;Individualised Learner Record&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Apprenticeships in</t>
   </si>
 </sst>
 </file>
@@ -1236,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49D33D53-EEC7-4B18-8C67-5F9034426AB5}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="25" style="6" customWidth="1"/>
@@ -2185,6 +2226,47 @@
         <v>149</v>
       </c>
       <c r="G24" s="8"/>
+    </row>
+    <row r="25" spans="1:13" ht="232.5" thickBot="1">
+      <c r="A25" t="s">
+        <v>219</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D25" t="s">
+        <v>228</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>227</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
Get app data working as it should in the local skills page
</commit_message>
<xml_diff>
--- a/Data/3-2_dataText/dataText.xlsx
+++ b/Data/3-2_dataText/dataText.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-2_dataText/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9250B018-2B86-44BF-9E5D-4DD6E1466454}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{50BC6191-9AF8-4D14-B309-FB400C7A4CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EA256D6-C674-4EEB-B0DB-876B1E2383E1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{E004AAF5-AC7D-409D-877C-9EBD23056743}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="229">
   <si>
     <t>inactiveRate</t>
   </si>
@@ -811,9 +811,6 @@
   </si>
   <si>
     <t>apprenticeships</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This indicator shows apprenticeship achievements. </t>
   </si>
   <si>
     <t>Include all age apprenticeships.
@@ -2234,38 +2231,36 @@
       <c r="B25" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="5"/>
+      <c r="D25" t="s">
+        <v>227</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G25" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F25" s="2" t="s">
+      <c r="H25" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="G25" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="H25" s="8" t="s">
+      <c r="I25" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="J25" s="8" t="s">
         <v>224</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>225</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>219</v>
       </c>
       <c r="L25" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="M25" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="M25" s="8" t="s">
-        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>